<commit_message>
ED Fig. 3f: persistence of the catalyst-level methanol changes under re-measurement
The main text cites ED Fig. 3 for the 63-comparison re-measurement (21.2 changes per draw, 17-26; 8 of the 10 above
5 % persist in >= 90 %), which panels a-e (81 point-level comparisons) did not show. Panel f plots each catalyst
change with more catalyst loaded and at laboratory conversion; page 183 x 244 mm, panels a-e moved up with their
tweak keys. Captions, Source Data and an audit lock updated; audit 362/0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/SourceData_EDFig3.xlsx
+++ b/source_data/SourceData_EDFig3.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="c" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="d" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="e" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="f" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -592,6 +593,42 @@
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>panel f</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>analysis/meoh_catalyst_level_robustness_2026_10_24/groups_noise_raised.csv, groups_noise_lab.csv, summary_noise_*.json; cost gap from analysis/meoh_catalyst_level_2026_10_19/groups_catalyst_level_conversion_raised.csv, groups_catalyst_level.csv</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>constants drawn on panel f</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>analysis/meoh_catalyst_level_robustness_2026_10_24/groups_noise_raised.csv,</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5459,4 +5496,1377 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>panel f</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>source: analysis/meoh_catalyst_level_robustness_2026_10_24/groups_noise_raised.csv, groups_noise_lab.csv, summary_noise_*.json; cost gap from analysis/meoh_catalyst_level_2026_10_19/groups_catalyst_level_conversion_raised.csv, groups_catalyst_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>doi</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>p_changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10.1016/j.jes.2023.05.010 | 30 bar | H2/CO2 4 | 18000 h-1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>10.1016/j.jes.2023.05.010</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.260292</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c06647 | 50 bar | H2/CO2 3 | 9 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c06647</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.207087</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.abi6012 | 40 bar | H2/CO2 3 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.abi6012</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.200049</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10.1038/s41467-026-72876-w | 20 bar | H2/CO2 3 | 450 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>10.1038/s41467-026-72876-w</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.190547</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h | 4 bar | H2/CO2 3.8 | 10.6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.144732</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c01275 | 50 bar | H2/CO2 3 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c01275</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.119568</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.abi6012 | 40 bar | H2/CO2 3 | 12 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.abi6012</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.112073</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.5c05984 | 100 bar | H2/CO2 4 | 10 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.5c05984</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.0585369</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.9b03305 | 50 bar | H2/CO2 4 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.9b03305</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.0120959</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.9675</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c06780 | 30 bar | H2/CO2 4 | 40 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c06780</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.0007154</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.9565</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.1c03170 | 30 bar | H2/CO2 3 | 60 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.1c03170</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.00684566</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c03987 | 14 bar | H2/CO2 3 | 30 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c03987</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.0614462</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.8815</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10.1038/s41557-026-02104-x | 50 bar | H2/CO2 3 | 1.5 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>10.1038/s41557-026-02104-x</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.00303501</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.8179999999999999</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.aea7041 | 50 bar | H2/CO2 4 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.aea7041</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.0131874</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.787</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10.1038/s41565-026-02135-y | 50 bar | H2/CO2 4 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>10.1038/s41565-026-02135-y</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2.40437e-06</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.6895</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10.1002/cctc.202000974 | 20 bar | H2/CO2 3 | 3.6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>10.1002/cctc.202000974</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.238666</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.6495</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10.1016/j.fuel.2024.131111 | 40 bar | H2/CO2 5 | 12 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>10.1016/j.fuel.2024.131111</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.0350789</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.593</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>10.1039/c5cy00372e | 50 bar | H2/CO2 3.04 | 10 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>10.1039/c5cy00372e</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.00390395</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.5575</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>10.1016/j.fuel.2023.127927 | 20 bar | H2/CO2 3 | 2.4 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10.1016/j.fuel.2023.127927</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0.00293911</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.552</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h | 360 bar | H2/CO2 3.8 | 10.6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0.0147289</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.485</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>more_catalyst</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c02907 | 5 bar | H2/CO2 3 | 30 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c02907</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0.00324908</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.426</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h | 100 bar | H2/CO2 3.8 | 10.6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1.57562</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c04842 | 30 bar | H2/CO2 2 | 48 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c04842</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0.364174</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10.1016/j.jes.2023.05.010 | 30 bar | H2/CO2 4 | 18000 h-1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10.1016/j.jes.2023.05.010</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.23079</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c04842 | 30 bar | H2/CO2 3 | 48 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c04842</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.178319</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.9b03305 | 50 bar | H2/CO2 4 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.9b03305</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>0.144612</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.abi6012 | 40 bar | H2/CO2 3 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.abi6012</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0.133089</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c06714 | 50 bar | H2/CO2 4 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c06714</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.0853284</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.abi6012 | 40 bar | H2/CO2 3 | 12 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.abi6012</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.0365433</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10.1039/c6ra28305e | 30 bar | H2/CO2 3 | 3600 h-1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>10.1039/c6ra28305e</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0.0264893</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10.1016/j.fuel.2024.131111 | 40 bar | H2/CO2 5 | 12 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>10.1016/j.fuel.2024.131111</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0.118529</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10.1016/j.cattod.2020.05.049 | 41 bar | H2/CO2 3 | 3.6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>10.1016/j.cattod.2020.05.049</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0.549488</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c03987 | 14 bar | H2/CO2 3 | 30 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c03987</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0.10111</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.991</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c01275 | 50 bar | H2/CO2 3 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c01275</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0.0738813</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.9825</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10.1016/j.jcat.2012.05.020 | 30 bar | H2/CO2 3 | 13.4 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>10.1016/j.jcat.2012.05.020</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0.376425</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.972</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.5c05984 | 100 bar | H2/CO2 4 | 10 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.5c05984</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.0667758</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.972</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.1c03170 | 30 bar | H2/CO2 3 | 60 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.1c03170</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0.628244</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10.1038/s41565-026-02135-y | 50 bar | H2/CO2 4 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10.1038/s41565-026-02135-y</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0.400722</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.9295</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c02907 | 20 bar | H2/CO2 3 | 30 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c02907</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0.07576919999999999</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.825</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.aea7041 | 50 bar | H2/CO2 4 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>10.1126/sciadv.aea7041</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0.376472</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.7865</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h | 360 bar | H2/CO2 3.8 | 10.6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0.0804754</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>10.1007/s11426-026-3904-1 | 20 bar | H2/CO2 3 | 6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>10.1007/s11426-026-3904-1</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0.00564525</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.9b01869 | 50 bar | H2/CO2 4 | 24000 h-1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.9b01869</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.0441059</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.666</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>10.1002/cctc.202000974 | 20 bar | H2/CO2 3 | 3.6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>10.1002/cctc.202000974</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.00633792</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.5935</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c02907 | 10 bar | H2/CO2 3 | 30 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>10.1021/acscatal.6c02907</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.09116009999999999</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.5565</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h | 30 bar | H2/CO2 3.8 | 10.6 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>10.1039/c2cy20604h</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.0202078</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.537</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>laboratory_conversion</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10.1016/j.fuel.2023.127927 | 20 bar | H2/CO2 3 | 2.4 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>10.1016/j.fuel.2023.127927</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0.00293911</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.5235</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>constants drawn on panel f</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>source: analysis/meoh_catalyst_level_robustness_2026_10_24/groups_noise_raised.csv,</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>more_catalyst.observed</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>more_catalyst.groups</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>more_catalyst.mean</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>21.2145</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>more_catalyst.q025</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>more_catalyst.q975</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>more_catalyst.kept90</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>more_catalyst.kept50</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>more_catalyst.gt5</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>more_catalyst.gt5_kept90</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.observed</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.groups</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.mean</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>25.147</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.q025</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.q975</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.kept90</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.kept50</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.gt5</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>laboratory_conversion.gt5_kept90</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>